<commit_message>
Add Samildol attendance sample records
</commit_message>
<xml_diff>
--- a/sample-data/아이돌 출퇴근 정보/Samildol_external_activity_records.xlsx
+++ b/sample-data/아이돌 출퇴근 정보/Samildol_external_activity_records.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="활동기록" sheetId="1" r:id="Rc1392303f1f240b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일정표" sheetId="2" r:id="R05c13ded5aef4d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="결제내역" sheetId="3" r:id="Ra29098a5829f47af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="활동기록" sheetId="1" r:id="R3a61dcc85f4448fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일정표" sheetId="2" r:id="R39295c0b26094adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="결제내역" sheetId="3" r:id="Rd96ce3197f124039"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +36,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -46,6 +46,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F7A8C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -69,7 +74,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -77,6 +82,18 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -687,6 +704,446 @@
         <x:v>콘서트 리허설</x:v>
       </x:c>
     </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="12" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="B21" s="11" t="str">
+        <x:v>Haru</x:v>
+      </x:c>
+      <x:c r="C21" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D21" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E21" s="11" t="str">
+        <x:v>ATT-20260711-001</x:v>
+      </x:c>
+      <x:c r="F21" s="11" t="str">
+        <x:v>팬미팅 연습 입실</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="12" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="str">
+        <x:v>Min</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="str">
+        <x:v>ATT-20260711-002</x:v>
+      </x:c>
+      <x:c r="F22" s="11" t="str">
+        <x:v>팬미팅 연습 입실</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="12" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="B23" s="11" t="str">
+        <x:v>Seo</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="str">
+        <x:v>ATT-20260711-003</x:v>
+      </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>팬미팅 연습 입실</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="12" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="str">
+        <x:v>Lia</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="str">
+        <x:v>ATT-20260711-004</x:v>
+      </x:c>
+      <x:c r="F24" s="11" t="str">
+        <x:v>팬미팅 연습 입실</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="12" t="n">
+        <x:v>46214</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="str">
+        <x:v>Noa</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>ATT-20260711-005</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>팬미팅 연습 입실</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="12" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="B26" s="11" t="str">
+        <x:v>Haru</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="D26" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="str">
+        <x:v>ATT-20260712-001</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>콘텐츠 촬영 대기</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="12" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>Seo</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="str">
+        <x:v>ATT-20260712-002</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>콘텐츠 촬영 대기</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="12" t="n">
+        <x:v>46215</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="str">
+        <x:v>Noa</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="str">
+        <x:v>대기</x:v>
+      </x:c>
+      <x:c r="D28" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="str">
+        <x:v>ATT-20260712-003</x:v>
+      </x:c>
+      <x:c r="F28" s="11" t="str">
+        <x:v>콘텐츠 촬영 대기</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="12" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B29" s="11" t="str">
+        <x:v>Haru</x:v>
+      </x:c>
+      <x:c r="C29" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D29" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="str">
+        <x:v>ATT-20260713-001</x:v>
+      </x:c>
+      <x:c r="F29" s="11" t="str">
+        <x:v>월간 콘텐츠 회의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="12" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B30" s="11" t="str">
+        <x:v>Min</x:v>
+      </x:c>
+      <x:c r="C30" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D30" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E30" s="11" t="str">
+        <x:v>ATT-20260713-002</x:v>
+      </x:c>
+      <x:c r="F30" s="11" t="str">
+        <x:v>월간 콘텐츠 회의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="12" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B31" s="11" t="str">
+        <x:v>Seo</x:v>
+      </x:c>
+      <x:c r="C31" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D31" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="str">
+        <x:v>ATT-20260713-003</x:v>
+      </x:c>
+      <x:c r="F31" s="11" t="str">
+        <x:v>월간 콘텐츠 회의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="12" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B32" s="11" t="str">
+        <x:v>Lia</x:v>
+      </x:c>
+      <x:c r="C32" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D32" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E32" s="11" t="str">
+        <x:v>ATT-20260713-004</x:v>
+      </x:c>
+      <x:c r="F32" s="11" t="str">
+        <x:v>월간 콘텐츠 회의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="12" t="n">
+        <x:v>46216</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="str">
+        <x:v>Noa</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="str">
+        <x:v>ATT-20260713-005</x:v>
+      </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>월간 콘텐츠 회의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="12" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="B34" s="11" t="str">
+        <x:v>Haru</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D34" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E34" s="11" t="str">
+        <x:v>ATT-20260714-001</x:v>
+      </x:c>
+      <x:c r="F34" s="11" t="str">
+        <x:v>보컬 퍼포먼스 점검</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="12" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="str">
+        <x:v>Min</x:v>
+      </x:c>
+      <x:c r="C35" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D35" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E35" s="11" t="str">
+        <x:v>ATT-20260714-002</x:v>
+      </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>보컬 퍼포먼스 점검</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="12" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="B36" s="11" t="str">
+        <x:v>Lia</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D36" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E36" s="11" t="str">
+        <x:v>ATT-20260714-003</x:v>
+      </x:c>
+      <x:c r="F36" s="11" t="str">
+        <x:v>보컬 퍼포먼스 점검</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="12" t="n">
+        <x:v>46217</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="str">
+        <x:v>Noa</x:v>
+      </x:c>
+      <x:c r="C37" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D37" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="str">
+        <x:v>ATT-20260714-004</x:v>
+      </x:c>
+      <x:c r="F37" s="11" t="str">
+        <x:v>보컬 퍼포먼스 점검</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="12" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B38" s="11" t="str">
+        <x:v>Haru</x:v>
+      </x:c>
+      <x:c r="C38" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D38" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E38" s="11" t="str">
+        <x:v>ATT-20260715-001</x:v>
+      </x:c>
+      <x:c r="F38" s="11" t="str">
+        <x:v>정산기간 마감 리허설</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="12" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B39" s="11" t="str">
+        <x:v>Min</x:v>
+      </x:c>
+      <x:c r="C39" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D39" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="str">
+        <x:v>ATT-20260715-002</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="str">
+        <x:v>정산기간 마감 리허설</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="12" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="str">
+        <x:v>Seo</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="str">
+        <x:v>ATT-20260715-003</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>정산기간 마감 리허설</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="12" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B41" s="11" t="str">
+        <x:v>Lia</x:v>
+      </x:c>
+      <x:c r="C41" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D41" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="str">
+        <x:v>ATT-20260715-004</x:v>
+      </x:c>
+      <x:c r="F41" s="11" t="str">
+        <x:v>정산기간 마감 리허설</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="12" t="n">
+        <x:v>46218</x:v>
+      </x:c>
+      <x:c r="B42" s="11" t="str">
+        <x:v>Noa</x:v>
+      </x:c>
+      <x:c r="C42" s="11" t="str">
+        <x:v>출근</x:v>
+      </x:c>
+      <x:c r="D42" s="11" t="str">
+        <x:v>회사 입출 기록</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="str">
+        <x:v>ATT-20260715-005</x:v>
+      </x:c>
+      <x:c r="F42" s="11" t="str">
+        <x:v>정산기간 마감 리허설</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>